<commit_message>
docs: improve final report for testing
</commit_message>
<xml_diff>
--- a/devlog/testing/general_test_table.xlsx
+++ b/devlog/testing/general_test_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\gitrepo\2026-group-5\devlog\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D5899EB-6715-4873-A5E0-CE093B40546E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCA316F5-0F1D-42BF-8B00-6FF840BD016E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="13665" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{9A71F247-E005-4031-B9D5-3D5AC84D32D3}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{9A71F247-E005-4031-B9D5-3D5AC84D32D3}"/>
   </bookViews>
   <sheets>
     <sheet name="SummaryTables" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="415">
   <si>
     <t>ID</t>
   </si>
@@ -431,9 +431,6 @@
     <t>Jinni-Li</t>
   </si>
   <si>
-    <t>Boundary Value</t>
-  </si>
-  <si>
     <t>End-state return flow behaved correctly.</t>
   </si>
   <si>
@@ -845,9 +842,6 @@
     <t>Input resets safely and the player does not continue moving after focus returns.</t>
   </si>
   <si>
-    <t>Boundary value</t>
-  </si>
-  <si>
     <t>BV06</t>
   </si>
   <si>
@@ -1005,9 +999,6 @@
   </si>
   <si>
     <t>Input Handling</t>
-  </si>
-  <si>
-    <t>Internal Logic</t>
   </si>
   <si>
     <t>WT08</t>
@@ -1352,6 +1343,12 @@
   </si>
   <si>
     <t>Yan Cui</t>
+  </si>
+  <si>
+    <t>BT - Boundary Value</t>
+  </si>
+  <si>
+    <t>Selected Internal Logic Areas</t>
   </si>
 </sst>
 </file>
@@ -1507,7 +1504,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="20" formatCode="d\-mmm\-yy"/>
+      <numFmt numFmtId="164" formatCode="d\-mmm\-yy"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
@@ -1539,7 +1536,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="20" formatCode="d\-mmm\-yy"/>
+      <numFmt numFmtId="164" formatCode="d\-mmm\-yy"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
@@ -1685,7 +1682,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="20" formatCode="d\-mmm\-yy"/>
+      <numFmt numFmtId="164" formatCode="d\-mmm\-yy"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1705,7 +1702,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="20" formatCode="d\-mmm\-yy"/>
+      <numFmt numFmtId="164" formatCode="d\-mmm\-yy"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1965,7 +1962,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jinni Li" refreshedDate="46131.988688078702" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="71" xr:uid="{E4CF02EB-9DA9-4FE9-B3FC-948C690D7CDB}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jinni Li" refreshedDate="46135.989701967592" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="71" xr:uid="{E4CF02EB-9DA9-4FE9-B3FC-948C690D7CDB}">
   <cacheSource type="worksheet">
     <worksheetSource name="Table2"/>
   </cacheSource>
@@ -1983,12 +1980,14 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="Group" numFmtId="0">
-      <sharedItems count="6">
+      <sharedItems count="8">
         <s v="Deployment and Platform Behaviour"/>
         <s v="Core Game Flow"/>
         <s v="Rendering, UI, and Audio"/>
         <s v="Player Interaction Systems"/>
-        <s v="Internal Logic"/>
+        <s v="Selected Internal Logic Areas"/>
+        <s v="Selected Internal Systems" u="1"/>
+        <s v="Internal Logic" u="1"/>
         <s v="AI and Gameplay Integration" u="1"/>
       </sharedItems>
     </cacheField>
@@ -2068,7 +2067,7 @@
   <r>
     <s v="BT04"/>
     <s v="Intro progression"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Tutorial / Story Flow"/>
     <x v="1"/>
     <s v="Enter key in intro state"/>
@@ -2185,7 +2184,7 @@
   <r>
     <s v="BT13"/>
     <s v="Screen scaling"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Rendering / UI"/>
     <x v="2"/>
     <s v="Window sizes: small / medium / large"/>
@@ -2718,7 +2717,7 @@
   <r>
     <s v="BV01"/>
     <s v="First Enter press"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Input Handling"/>
     <x v="3"/>
     <s v="First Enter press"/>
@@ -2731,7 +2730,7 @@
   <r>
     <s v="BV02"/>
     <s v="Very small window"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Rendering / UI"/>
     <x v="2"/>
     <s v="Very small window"/>
@@ -2744,7 +2743,7 @@
   <r>
     <s v="BV03"/>
     <s v="Very large window"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Rendering / UI"/>
     <x v="2"/>
     <s v="Very large window"/>
@@ -2757,7 +2756,7 @@
   <r>
     <s v="BV04"/>
     <s v="Rapid key presses"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Loot / Inventory"/>
     <x v="3"/>
     <s v="Rapid repeated Enter input"/>
@@ -2770,7 +2769,7 @@
   <r>
     <s v="BV05"/>
     <s v="Asset loading delay"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Deployment &amp; Launch"/>
     <x v="0"/>
     <s v="Initial asset loading"/>
@@ -2783,7 +2782,7 @@
   <r>
     <s v="BV06"/>
     <s v="Tutorial skip hold threshold"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Tutorial / Story Flow"/>
     <x v="1"/>
     <s v="hold E for less than 0.8s / at least 0.8s"/>
@@ -2796,7 +2795,7 @@
   <r>
     <s v="BV07"/>
     <s v="Playthrough unlock hold threshold"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Tutorial / Story Flow"/>
     <x v="1"/>
     <s v="hold E for less than 1.2s / at least 1.2s"/>
@@ -2809,7 +2808,7 @@
   <r>
     <s v="BV08"/>
     <s v="Rapid repeated door input"/>
-    <s v="Boundary Value"/>
+    <s v="BT - Boundary Value"/>
     <s v="Doors / Objectives"/>
     <x v="3"/>
     <s v="spam E around door cooldown"/>
@@ -2823,7 +2822,7 @@
     <s v="WT01"/>
     <s v="setGameState logic"/>
     <s v="White-box"/>
-    <s v="Internal Logic"/>
+    <s v="Selected Internal Logic Areas"/>
     <x v="4"/>
     <s v="State transition logic"/>
     <s v="Call or trace setGameState with valid transitions."/>
@@ -2836,7 +2835,7 @@
     <s v="WT02"/>
     <s v="Screen routing logic"/>
     <s v="White-box"/>
-    <s v="Internal Logic"/>
+    <s v="Selected Internal Logic Areas"/>
     <x v="4"/>
     <s v="start -&gt; tutorial/difficulty / intro -&gt; playing or map select / ending follow-up"/>
     <s v="Trace the screen handlers and screen-manager routing for each major branch."/>
@@ -2875,7 +2874,7 @@
     <s v="WT05"/>
     <s v="Layout helper values"/>
     <s v="White-box"/>
-    <s v="Internal Logic"/>
+    <s v="Selected Internal Logic Areas"/>
     <x v="4"/>
     <s v="Layout helper outputs"/>
     <s v="Run layout or scaling helper functions with different sizes."/>
@@ -2888,7 +2887,7 @@
     <s v="WT06"/>
     <s v="Overlay draw conditions"/>
     <s v="White-box"/>
-    <s v="Internal Logic"/>
+    <s v="Selected Internal Logic Areas"/>
     <x v="4"/>
     <s v="Overlay render guard"/>
     <s v="Trace overlay rendering for different states."/>
@@ -2901,7 +2900,7 @@
     <s v="WT07"/>
     <s v="Interaction prompt priority"/>
     <s v="White-box"/>
-    <s v="Internal Logic"/>
+    <s v="Selected Internal Logic Areas"/>
     <x v="4"/>
     <s v="exit &gt; chest &gt; door &gt; button"/>
     <s v="Trace getInteractionPrompt() with overlapping nearby interactables."/>
@@ -2940,7 +2939,7 @@
     <s v="WT10"/>
     <s v="Input resolution and reset"/>
     <s v="White-box"/>
-    <s v="Internal Logic"/>
+    <s v="Selected Internal Logic Areas"/>
     <x v="4"/>
     <s v="last-pressed axis / interact consume / blur reset"/>
     <s v="Trace InputSystem with opposing directions, interact presses, and reset calls."/>
@@ -3014,13 +3013,15 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
-      <items count="7">
+      <items count="9">
         <item x="1"/>
         <item x="0"/>
-        <item x="4"/>
+        <item m="1" x="6"/>
         <item x="3"/>
         <item x="2"/>
+        <item m="1" x="7"/>
         <item m="1" x="5"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -3050,13 +3051,13 @@
       <x v="1"/>
     </i>
     <i>
-      <x v="2"/>
-    </i>
-    <i>
       <x v="3"/>
     </i>
     <i>
       <x v="4"/>
+    </i>
+    <i>
+      <x v="7"/>
     </i>
     <i t="grand">
       <x/>
@@ -3440,8 +3441,8 @@
   <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.46484375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.86328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
@@ -3454,15 +3455,15 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B3" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" s="11" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B4" s="15">
         <v>27</v>
@@ -3470,7 +3471,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" s="11" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B5" s="15">
         <v>4</v>
@@ -3478,31 +3479,31 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>318</v>
+        <v>348</v>
       </c>
       <c r="B6" s="15">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" s="11" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="B7" s="15">
-        <v>24</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" s="11" t="s">
-        <v>348</v>
+        <v>414</v>
       </c>
       <c r="B8" s="15">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" s="11" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B9" s="15">
         <v>71</v>
@@ -3510,10 +3511,10 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24" s="10" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="B24" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.45">
@@ -3526,7 +3527,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A26" s="11" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B26" s="15">
         <v>71</v>
@@ -3567,10 +3568,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>3</v>
@@ -3605,10 +3606,10 @@
         <v>102</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>10</v>
@@ -3626,7 +3627,7 @@
         <v>46098</v>
       </c>
       <c r="K2" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>12</v>
@@ -3643,10 +3644,10 @@
         <v>102</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>15</v>
@@ -3664,7 +3665,7 @@
         <v>46098</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>112</v>
@@ -3681,10 +3682,10 @@
         <v>102</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>19</v>
@@ -3702,7 +3703,7 @@
         <v>46098</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>113</v>
@@ -3716,13 +3717,13 @@
         <v>22</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>126</v>
+        <v>413</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>23</v>
@@ -3740,7 +3741,7 @@
         <v>46098</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>56</v>
@@ -3757,10 +3758,10 @@
         <v>102</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>27</v>
@@ -3778,7 +3779,7 @@
         <v>46098</v>
       </c>
       <c r="K6" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="27" x14ac:dyDescent="0.45">
@@ -3792,10 +3793,10 @@
         <v>102</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>31</v>
@@ -3813,7 +3814,7 @@
         <v>46098</v>
       </c>
       <c r="K7" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="40.5" x14ac:dyDescent="0.45">
@@ -3827,10 +3828,10 @@
         <v>102</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>35</v>
@@ -3848,7 +3849,7 @@
         <v>46127</v>
       </c>
       <c r="K8" s="13" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="54" x14ac:dyDescent="0.45">
@@ -3856,25 +3857,25 @@
         <v>38</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F9" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>129</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>130</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>12</v>
@@ -3883,7 +3884,7 @@
         <v>46128</v>
       </c>
       <c r="K9" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="27" x14ac:dyDescent="0.45">
@@ -3897,10 +3898,10 @@
         <v>102</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>40</v>
@@ -3918,7 +3919,7 @@
         <v>46098</v>
       </c>
       <c r="K10" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="27" x14ac:dyDescent="0.45">
@@ -3932,10 +3933,10 @@
         <v>102</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>45</v>
@@ -3953,7 +3954,7 @@
         <v>46098</v>
       </c>
       <c r="K11" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="40.15" customHeight="1" x14ac:dyDescent="0.45">
@@ -3967,10 +3968,10 @@
         <v>102</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>49</v>
@@ -3988,33 +3989,33 @@
         <v>46098</v>
       </c>
       <c r="K12" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F13" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>135</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>12</v>
@@ -4023,10 +4024,10 @@
         <v>46129</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="27" x14ac:dyDescent="0.45">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>57</v>
       </c>
@@ -4034,13 +4035,13 @@
         <v>52</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>126</v>
+        <v>413</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>53</v>
@@ -4058,12 +4059,12 @@
         <v>46127</v>
       </c>
       <c r="K14" s="13" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>58</v>
@@ -4072,10 +4073,10 @@
         <v>102</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>59</v>
@@ -4093,12 +4094,12 @@
         <v>46127</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>58</v>
@@ -4107,19 +4108,19 @@
         <v>102</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F16" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="H16" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>137</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>12</v>
@@ -4128,33 +4129,33 @@
         <v>46128</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F17" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="H17" s="5" t="s">
         <v>140</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>141</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>12</v>
@@ -4163,33 +4164,33 @@
         <v>46128</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A18" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F18" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="H18" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>12</v>
@@ -4198,33 +4199,33 @@
         <v>46128</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A19" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F19" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="5" t="s">
         <v>149</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>150</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>12</v>
@@ -4233,33 +4234,33 @@
         <v>46128</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F20" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="G20" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="H20" s="5" t="s">
         <v>154</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>155</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>12</v>
@@ -4268,33 +4269,33 @@
         <v>46128</v>
       </c>
       <c r="K20" s="13" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="54" x14ac:dyDescent="0.45">
       <c r="A21" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F21" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="H21" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>12</v>
@@ -4303,33 +4304,33 @@
         <v>46128</v>
       </c>
       <c r="K21" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F22" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="H22" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>163</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>12</v>
@@ -4338,33 +4339,33 @@
         <v>46128</v>
       </c>
       <c r="K22" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A23" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F23" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="G23" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="H23" s="5" t="s">
         <v>167</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>168</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>12</v>
@@ -4373,33 +4374,33 @@
         <v>46128</v>
       </c>
       <c r="K23" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="36.4" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F24" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="H24" s="5" t="s">
         <v>171</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>172</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>12</v>
@@ -4408,33 +4409,33 @@
         <v>46128</v>
       </c>
       <c r="K24" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="67.5" x14ac:dyDescent="0.45">
       <c r="A25" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F25" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="H25" s="5" t="s">
         <v>175</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>176</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>12</v>
@@ -4443,33 +4444,33 @@
         <v>46128</v>
       </c>
       <c r="K25" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A26" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F26" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="G26" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="G26" s="5" t="s">
+      <c r="H26" s="5" t="s">
         <v>180</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>181</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>12</v>
@@ -4478,33 +4479,33 @@
         <v>46127</v>
       </c>
       <c r="K26" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F27" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="H27" s="5" t="s">
         <v>185</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>186</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>12</v>
@@ -4513,33 +4514,33 @@
         <v>46127</v>
       </c>
       <c r="K27" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F28" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="H28" s="5" t="s">
         <v>189</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>190</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>12</v>
@@ -4548,33 +4549,33 @@
         <v>46128</v>
       </c>
       <c r="K28" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F29" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="H29" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>194</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>12</v>
@@ -4583,33 +4584,33 @@
         <v>46128</v>
       </c>
       <c r="K29" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A30" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F30" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="G30" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="G30" s="5" t="s">
+      <c r="H30" s="5" t="s">
         <v>198</v>
-      </c>
-      <c r="H30" s="5" t="s">
-        <v>199</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>12</v>
@@ -4618,33 +4619,33 @@
         <v>46128</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A31" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F31" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="H31" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>203</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>12</v>
@@ -4653,33 +4654,33 @@
         <v>46128</v>
       </c>
       <c r="K31" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A32" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F32" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="H32" s="5" t="s">
         <v>206</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>207</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>12</v>
@@ -4688,33 +4689,33 @@
         <v>46128</v>
       </c>
       <c r="K32" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A33" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F33" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="H33" s="5" t="s">
         <v>210</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>211</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>12</v>
@@ -4723,33 +4724,33 @@
         <v>46128</v>
       </c>
       <c r="K33" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="54" x14ac:dyDescent="0.45">
       <c r="A34" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>12</v>
@@ -4758,33 +4759,33 @@
         <v>46128</v>
       </c>
       <c r="K34" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A35" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F35" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="H35" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>12</v>
@@ -4793,33 +4794,33 @@
         <v>46128</v>
       </c>
       <c r="K35" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A36" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F36" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="H36" s="5" t="s">
         <v>221</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>222</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>12</v>
@@ -4828,33 +4829,33 @@
         <v>46128</v>
       </c>
       <c r="K36" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A37" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F37" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="G37" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="G37" s="5" t="s">
+      <c r="H37" s="5" t="s">
         <v>226</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>227</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>12</v>
@@ -4863,33 +4864,33 @@
         <v>46129</v>
       </c>
       <c r="K37" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A38" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F38" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="H38" s="5" t="s">
         <v>230</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>231</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>12</v>
@@ -4898,33 +4899,33 @@
         <v>46128</v>
       </c>
       <c r="K38" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="54" x14ac:dyDescent="0.45">
       <c r="A39" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F39" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="H39" s="5" t="s">
         <v>234</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>235</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>12</v>
@@ -4933,33 +4934,33 @@
         <v>46128</v>
       </c>
       <c r="K39" s="13" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A40" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F40" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="G40" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="G40" s="5" t="s">
+      <c r="H40" s="5" t="s">
         <v>240</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>241</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>12</v>
@@ -4968,33 +4969,33 @@
         <v>46128</v>
       </c>
       <c r="K40" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A41" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F41" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="G41" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="G41" s="5" t="s">
+      <c r="H41" s="5" t="s">
         <v>245</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>246</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>12</v>
@@ -5003,33 +5004,33 @@
         <v>46128</v>
       </c>
       <c r="K41" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A42" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F42" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="H42" s="5" t="s">
         <v>249</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>341</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>250</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>12</v>
@@ -5038,33 +5039,33 @@
         <v>46128</v>
       </c>
       <c r="K42" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A43" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F43" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="G43" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="G43" s="5" t="s">
+      <c r="H43" s="5" t="s">
         <v>254</v>
-      </c>
-      <c r="H43" s="5" t="s">
-        <v>255</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>12</v>
@@ -5073,33 +5074,33 @@
         <v>46129</v>
       </c>
       <c r="K43" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A44" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F44" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>258</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>259</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>12</v>
@@ -5108,33 +5109,33 @@
         <v>46128</v>
       </c>
       <c r="K44" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A45" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F45" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="H45" s="5" t="s">
         <v>262</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="H45" s="5" t="s">
-        <v>263</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>12</v>
@@ -5143,33 +5144,33 @@
         <v>46128</v>
       </c>
       <c r="K45" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A46" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D46" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="H46" s="5" t="s">
         <v>361</v>
-      </c>
-      <c r="E46" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>364</v>
       </c>
       <c r="I46" s="5" t="s">
         <v>12</v>
@@ -5178,33 +5179,33 @@
         <v>46128</v>
       </c>
       <c r="K46" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A47" s="5" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>12</v>
@@ -5213,33 +5214,33 @@
         <v>46128</v>
       </c>
       <c r="K47" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A48" s="5" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>12</v>
@@ -5248,33 +5249,33 @@
         <v>46128</v>
       </c>
       <c r="K48" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A49" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="I49" s="5" t="s">
         <v>12</v>
@@ -5283,33 +5284,33 @@
         <v>46128</v>
       </c>
       <c r="K49" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A50" s="5" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="I50" s="5" t="s">
         <v>12</v>
@@ -5318,33 +5319,33 @@
         <v>46128</v>
       </c>
       <c r="K50" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A51" s="5" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="I51" s="5" t="s">
         <v>12</v>
@@ -5353,33 +5354,33 @@
         <v>46128</v>
       </c>
       <c r="K51" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A52" s="5" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="I52" s="5" t="s">
         <v>12</v>
@@ -5388,33 +5389,33 @@
         <v>46128</v>
       </c>
       <c r="K52" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A53" s="5" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="I53" s="5" t="s">
         <v>12</v>
@@ -5423,33 +5424,33 @@
         <v>46128</v>
       </c>
       <c r="K53" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A54" s="5" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="I54" s="5" t="s">
         <v>12</v>
@@ -5458,10 +5459,10 @@
         <v>46128</v>
       </c>
       <c r="K54" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="27" x14ac:dyDescent="0.45">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A55" s="5" t="s">
         <v>62</v>
       </c>
@@ -5469,13 +5470,13 @@
         <v>63</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>126</v>
+        <v>413</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F55" s="5" t="s">
         <v>63</v>
@@ -5493,10 +5494,10 @@
         <v>46098</v>
       </c>
       <c r="K55" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="27" x14ac:dyDescent="0.45">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A56" s="5" t="s">
         <v>65</v>
       </c>
@@ -5504,13 +5505,13 @@
         <v>66</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>126</v>
+        <v>413</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F56" s="5" t="s">
         <v>66</v>
@@ -5528,24 +5529,24 @@
         <v>46127</v>
       </c>
       <c r="K56" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="27" x14ac:dyDescent="0.45">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A57" s="5" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>69</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>126</v>
+        <v>413</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F57" s="5" t="s">
         <v>69</v>
@@ -5563,10 +5564,10 @@
         <v>46127</v>
       </c>
       <c r="K57" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="27" x14ac:dyDescent="0.45">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A58" s="5" t="s">
         <v>72</v>
       </c>
@@ -5574,13 +5575,13 @@
         <v>73</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>126</v>
+        <v>413</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F58" s="5" t="s">
         <v>74</v>
@@ -5598,24 +5599,24 @@
         <v>46098</v>
       </c>
       <c r="K58" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="54" x14ac:dyDescent="0.45">
       <c r="A59" s="5" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>77</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>126</v>
+        <v>413</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F59" s="5" t="s">
         <v>78</v>
@@ -5633,33 +5634,33 @@
         <v>46127</v>
       </c>
       <c r="K59" s="13" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="27" x14ac:dyDescent="0.45">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A60" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="B60" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="C60" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="G60" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="C60" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="F60" s="5" t="s">
+      <c r="H60" s="5" t="s">
         <v>268</v>
-      </c>
-      <c r="G60" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="H60" s="5" t="s">
-        <v>270</v>
       </c>
       <c r="I60" s="5" t="s">
         <v>12</v>
@@ -5668,33 +5669,33 @@
         <v>46127</v>
       </c>
       <c r="K60" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A61" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B61" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="G61" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="H61" s="5" t="s">
         <v>271</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="F61" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="G61" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="H61" s="5" t="s">
-        <v>273</v>
       </c>
       <c r="I61" s="5" t="s">
         <v>12</v>
@@ -5703,33 +5704,33 @@
         <v>46127</v>
       </c>
       <c r="K61" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="27" x14ac:dyDescent="0.45">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A62" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="B62" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="F62" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="G62" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="H62" s="5" t="s">
         <v>274</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="D62" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="E62" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="F62" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="G62" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="H62" s="5" t="s">
-        <v>276</v>
       </c>
       <c r="I62" s="5" t="s">
         <v>12</v>
@@ -5738,10 +5739,10 @@
         <v>46128</v>
       </c>
       <c r="K62" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.45">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A63" s="5" t="s">
         <v>81</v>
       </c>
@@ -5752,10 +5753,10 @@
         <v>83</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="F63" s="5" t="s">
         <v>84</v>
@@ -5773,7 +5774,7 @@
         <v>46128</v>
       </c>
       <c r="K63" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="54" x14ac:dyDescent="0.45">
@@ -5781,25 +5782,25 @@
         <v>87</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="F64" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="G64" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="H64" s="5" t="s">
         <v>278</v>
-      </c>
-      <c r="G64" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="H64" s="5" t="s">
-        <v>280</v>
       </c>
       <c r="I64" s="5" t="s">
         <v>12</v>
@@ -5808,7 +5809,7 @@
         <v>46128</v>
       </c>
       <c r="K64" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="27" x14ac:dyDescent="0.45">
@@ -5822,10 +5823,10 @@
         <v>83</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F65" s="5" t="s">
         <v>89</v>
@@ -5843,7 +5844,7 @@
         <v>46129</v>
       </c>
       <c r="K65" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
@@ -5851,25 +5852,25 @@
         <v>97</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F66" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="H66" s="5" t="s">
         <v>282</v>
-      </c>
-      <c r="G66" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="H66" s="5" t="s">
-        <v>284</v>
       </c>
       <c r="I66" s="5" t="s">
         <v>12</v>
@@ -5878,12 +5879,12 @@
         <v>46129</v>
       </c>
       <c r="K66" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A67" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>93</v>
@@ -5892,10 +5893,10 @@
         <v>83</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="F67" s="5" t="s">
         <v>94</v>
@@ -5913,12 +5914,12 @@
         <v>46128</v>
       </c>
       <c r="K67" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="68" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A68" s="5" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>98</v>
@@ -5927,10 +5928,10 @@
         <v>83</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="F68" s="5" t="s">
         <v>99</v>
@@ -5948,33 +5949,33 @@
         <v>46129</v>
       </c>
       <c r="K68" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A69" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C69" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="F69" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="H69" s="5" t="s">
         <v>286</v>
-      </c>
-      <c r="G69" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="H69" s="5" t="s">
-        <v>288</v>
       </c>
       <c r="I69" s="5" t="s">
         <v>12</v>
@@ -5983,33 +5984,33 @@
         <v>46129</v>
       </c>
       <c r="K69" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="70" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A70" s="5" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F70" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="G70" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="H70" s="5" t="s">
         <v>291</v>
-      </c>
-      <c r="G70" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="H70" s="5" t="s">
-        <v>293</v>
       </c>
       <c r="I70" s="5" t="s">
         <v>12</v>
@@ -6018,33 +6019,33 @@
         <v>46129</v>
       </c>
       <c r="K70" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="71" spans="1:11" ht="27" x14ac:dyDescent="0.45">
       <c r="A71" s="5" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C71" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F71" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="G71" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="H71" s="5" t="s">
         <v>295</v>
-      </c>
-      <c r="G71" s="5" t="s">
-        <v>296</v>
-      </c>
-      <c r="H71" s="5" t="s">
-        <v>297</v>
       </c>
       <c r="I71" s="5" t="s">
         <v>12</v>
@@ -6053,33 +6054,33 @@
         <v>46131</v>
       </c>
       <c r="K71" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="72" spans="1:11" ht="40.5" x14ac:dyDescent="0.45">
       <c r="A72" s="5" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C72" s="5" t="s">
         <v>83</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>318</v>
+        <v>414</v>
       </c>
       <c r="F72" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="H72" s="5" t="s">
         <v>300</v>
-      </c>
-      <c r="G72" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="H72" s="5" t="s">
-        <v>302</v>
       </c>
       <c r="I72" s="5" t="s">
         <v>12</v>
@@ -6088,7 +6089,7 @@
         <v>46131</v>
       </c>
       <c r="K72" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>
@@ -6137,10 +6138,10 @@
         <v>120</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="43.15" thickBot="1" x14ac:dyDescent="0.5">
@@ -6157,7 +6158,7 @@
         <v>122</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>125</v>
@@ -6171,22 +6172,22 @@
     </row>
     <row r="3" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>122</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="G3" s="3">
         <v>46128</v>

</xml_diff>